<commit_message>
fix: corrigir fonte de dados do pipeline e regerar agregados
O pipeline lia data/resultados.csv (local, dez/2025, em rates) e dividia
por total_time de novo, gerando TPS ~70x menor que o real nos cenários
paralelos. Apontado para sysbench/results/aws/resultados.csv (jan/2026,
em contagens brutas) e adicionado drop_duplicates() em prepare_agg.

Inclui PNGs paralelos regerados, degradação atualizada (CSV+XLSX) e
prompt de regeneração para futuras trocas de fonte.
</commit_message>
<xml_diff>
--- a/graphics/data/degradacao.xlsx
+++ b/graphics/data/degradacao.xlsx
@@ -621,22 +621,22 @@
         </is>
       </c>
       <c r="D3" s="2" t="n">
-        <v>6.357966679524853</v>
+        <v>438.2316751147406</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>8.187255358337037</v>
+        <v>324.9178903525085</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>5.277055941122306</v>
+        <v>237.9404848812804</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>350.558</v>
+        <v>277.896</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>262.724</v>
+        <v>480.347</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>403.298</v>
+        <v>480.257</v>
       </c>
       <c r="J3" s="2">
         <f>IFERROR((E3-D3)/D3*100,"")</f>
@@ -755,22 +755,22 @@
         </is>
       </c>
       <c r="D5" s="2" t="n">
-        <v>3.778444437919872</v>
+        <v>183.8368805412824</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>5.37177321700913</v>
+        <v>161.424099717377</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>4.701507051537705</v>
+        <v>140.3036482289279</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>541.672</v>
+        <v>415.975</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>304.452</v>
+        <v>419.8729999999999</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>326.048</v>
+        <v>497.753</v>
       </c>
       <c r="J5" s="2">
         <f>IFERROR((E5-D5)/D5*100,"")</f>
@@ -889,22 +889,22 @@
         </is>
       </c>
       <c r="D7" s="2" t="n">
-        <v>26.87905709745969</v>
+        <v>1160.466987381118</v>
       </c>
       <c r="E7" s="2" t="n">
-        <v>27.3179245376038</v>
+        <v>887.6702484744052</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>12.57303403947906</v>
+        <v>928.5359421509012</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>55.82000000000001</v>
+        <v>145.863</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>87.88</v>
+        <v>205.965</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>185.232</v>
+        <v>207.078</v>
       </c>
       <c r="J7" s="2">
         <f>IFERROR((E7-D7)/D7*100,"")</f>
@@ -1023,22 +1023,22 @@
         </is>
       </c>
       <c r="D9" s="2" t="n">
-        <v>61.87179437940306</v>
+        <v>3721.733294272499</v>
       </c>
       <c r="E9" s="2" t="n">
-        <v>74.58109366741637</v>
+        <v>2182.301233671341</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>28.27072440075205</v>
+        <v>975.931796287108</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>61.54</v>
+        <v>35.981</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>47.992</v>
+        <v>144.574</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>80.32000000000001</v>
+        <v>242.555</v>
       </c>
       <c r="J9" s="2">
         <f>IFERROR((E9-D9)/D9*100,"")</f>
@@ -1157,22 +1157,22 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>0.2302886703637565</v>
+        <v>43.00333333333334</v>
       </c>
       <c r="E11" s="2" t="n">
-        <v>0.1761364837015759</v>
+        <v>42.13833333333334</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>0.2698615397080589</v>
+        <v>38.945</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>14415.256</v>
+        <v>1835.81</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>12346.346</v>
+        <v>1832.452</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>10090.23</v>
+        <v>1991.275</v>
       </c>
       <c r="J11" s="2">
         <f>IFERROR((E11-D11)/D11*100,"")</f>
@@ -1291,22 +1291,22 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>0.2538060254942948</v>
+        <v>20.23166666666667</v>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.2354181947131711</v>
+        <v>19.8</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>0.5274819757954763</v>
+        <v>19.945</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>3883.866</v>
+        <v>4406.449000000001</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>4203.93</v>
+        <v>4493.711</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>1924.324</v>
+        <v>4366.149</v>
       </c>
       <c r="J13" s="2">
         <f>IFERROR((E13-D13)/D13*100,"")</f>
@@ -1425,22 +1425,22 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>0.852373202258943</v>
+        <v>186.855</v>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0.7645924307652432</v>
+        <v>166.9383333333333</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>0.963442215407898</v>
+        <v>166.315</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>1917.53</v>
+        <v>612.29</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>3537.168</v>
+        <v>682.475</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>2662.186</v>
+        <v>634.8430000000001</v>
       </c>
       <c r="J15" s="2">
         <f>IFERROR((E15-D15)/D15*100,"")</f>
@@ -1559,22 +1559,22 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>4.401653601861566</v>
+        <v>348.8466666666667</v>
       </c>
       <c r="E17" s="2" t="n">
-        <v>2.699882141979113</v>
+        <v>274.9866666666667</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>1.324842648896007</v>
+        <v>302.7016666666667</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>349.08</v>
+        <v>407.564</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>667.4979999999999</v>
+        <v>483.59</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>2796.3</v>
+        <v>458.99</v>
       </c>
       <c r="J17" s="2">
         <f>IFERROR((E17-D17)/D17*100,"")</f>

</xml_diff>

<commit_message>
chore: regerar gráficos e degradação a partir do agg do fork rbizarrias@8bd96b8
Substituído data/resultados_agg.csv pelo conteúdo do fork rbizarrias
(commit 8bd96b8c). Principal diferença: Vitess READ Sequencial em
100K passa de 3.619 para 143 TPS, eliminando o "colapso" aparente —
o perfil de leitura vira essencialmente estável (-11% TPS / +12% Lat).
MySQL inalterado.
</commit_message>
<xml_diff>
--- a/graphics/data/degradacao.xlsx
+++ b/graphics/data/degradacao.xlsx
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="D11" s="2" t="n">
-        <v>43.00333333333334</v>
+        <v>43.79665300546448</v>
       </c>
       <c r="E11" s="2" t="n">
         <v>42.13833333333334</v>
@@ -1166,7 +1166,7 @@
         <v>38.945</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>1835.81</v>
+        <v>2027.676</v>
       </c>
       <c r="H11" s="2" t="n">
         <v>1832.452</v>
@@ -1224,7 +1224,7 @@
         </is>
       </c>
       <c r="D12" s="2" t="n">
-        <v>3619.392313533883</v>
+        <v>143.2916666666667</v>
       </c>
       <c r="E12" s="2" t="n">
         <v>91.02</v>
@@ -1233,7 +1233,7 @@
         <v>127.64</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>35.938</v>
+        <v>589.607</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>1006.02</v>
@@ -1291,7 +1291,7 @@
         </is>
       </c>
       <c r="D13" s="2" t="n">
-        <v>20.23166666666667</v>
+        <v>19.82083333333333</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>19.8</v>
@@ -1300,7 +1300,7 @@
         <v>19.945</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>4406.449000000001</v>
+        <v>4503.744000000001</v>
       </c>
       <c r="H13" s="2" t="n">
         <v>4493.711</v>
@@ -1425,7 +1425,7 @@
         </is>
       </c>
       <c r="D15" s="2" t="n">
-        <v>186.855</v>
+        <v>177.9841666666667</v>
       </c>
       <c r="E15" s="2" t="n">
         <v>166.9383333333333</v>
@@ -1434,7 +1434,7 @@
         <v>166.315</v>
       </c>
       <c r="G15" s="2" t="n">
-        <v>612.29</v>
+        <v>704.629</v>
       </c>
       <c r="H15" s="2" t="n">
         <v>682.475</v>
@@ -1495,7 +1495,7 @@
         <v>3159.365</v>
       </c>
       <c r="E16" s="2" t="n">
-        <v>1376.766666666667</v>
+        <v>1078.8325</v>
       </c>
       <c r="F16" s="2" t="n">
         <v>1037.568333333333</v>
@@ -1504,7 +1504,7 @@
         <v>41.486</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>111.552</v>
+        <v>133.0385</v>
       </c>
       <c r="I16" s="2" t="n">
         <v>107.459</v>
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="D17" s="2" t="n">
-        <v>348.8466666666667</v>
+        <v>315.9633333333333</v>
       </c>
       <c r="E17" s="2" t="n">
         <v>274.9866666666667</v>
@@ -1568,7 +1568,7 @@
         <v>302.7016666666667</v>
       </c>
       <c r="G17" s="2" t="n">
-        <v>407.564</v>
+        <v>475.1085</v>
       </c>
       <c r="H17" s="2" t="n">
         <v>483.59</v>

</xml_diff>